<commit_message>
pared down code, renamed constants
</commit_message>
<xml_diff>
--- a/data/_materials.xlsx
+++ b/data/_materials.xlsx
@@ -15020,10 +15020,10 @@
         <v>41236.755</v>
       </c>
       <c r="C249">
-        <v>4675.343999999999</v>
+        <v>4675.344</v>
       </c>
       <c r="D249">
-        <v>3477.663999999999</v>
+        <v>3477.664</v>
       </c>
       <c r="E249">
         <v>1197.68</v>
@@ -16052,7 +16052,7 @@
         <v>1738.8</v>
       </c>
       <c r="E276">
-        <v>586.3399999999999</v>
+        <v>586.34</v>
       </c>
       <c r="F276">
         <v>10000</v>
@@ -16654,10 +16654,10 @@
         <v>52189.691</v>
       </c>
       <c r="C292">
-        <v>4689.143999999999</v>
+        <v>4689.144</v>
       </c>
       <c r="D292">
-        <v>3481.463999999999</v>
+        <v>3481.464</v>
       </c>
       <c r="E292">
         <v>1207.68</v>
@@ -17338,10 +17338,10 @@
         <v>74645.507</v>
       </c>
       <c r="C310">
-        <v>9350.687999999998</v>
+        <v>9350.688</v>
       </c>
       <c r="D310">
-        <v>6955.327999999999</v>
+        <v>6955.328</v>
       </c>
       <c r="E310">
         <v>2395.36</v>
@@ -18142,7 +18142,7 @@
         <v>1738.8</v>
       </c>
       <c r="E331">
-        <v>586.3399999999999</v>
+        <v>586.34</v>
       </c>
       <c r="F331">
         <v>10000</v>
@@ -49679,7 +49679,7 @@
         <v>4675.28</v>
       </c>
       <c r="D1161">
-        <v>3477.6</v>
+        <v>3477.599999999999</v>
       </c>
       <c r="E1161">
         <v>1197.68</v>

</xml_diff>